<commit_message>
fix: Update OJT Practicum subject type and add prerequisite in curriculum
</commit_message>
<xml_diff>
--- a/BSIT-Curriculum (Major Only).xlsx
+++ b/BSIT-Curriculum (Major Only).xlsx
@@ -1207,10 +1207,10 @@
         <v>3</v>
       </c>
       <c r="F35" t="str">
-        <v>Major without Lab</v>
+        <v>Practicum/OJT</v>
       </c>
       <c r="G35" t="str">
-        <v>None</v>
+        <v>CAPS102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>